<commit_message>
Refine public summaries and spectral gradient docs
</commit_message>
<xml_diff>
--- a/analysis_outputs/all_anomaly_summary_tables/summary_tables.xlsx
+++ b/analysis_outputs/all_anomaly_summary_tables/summary_tables.xlsx
@@ -3252,7 +3252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3308,15 +3308,10 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>m50db</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
         <is>
           <t>result_source</t>
         </is>
@@ -3345,7 +3340,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -3366,14 +3361,11 @@
         <v>81.97</v>
       </c>
       <c r="K2" t="n">
-        <v>60.46</v>
-      </c>
-      <c r="L2" t="n">
-        <v>86.372</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>92.84999999999999</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; public-normal m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3392,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -3421,14 +3413,11 @@
         <v>98.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>87.77</v>
-      </c>
-      <c r="L3" t="n">
-        <v>97.33199999999999</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>99.7225</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; public-normal m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3444,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -3476,14 +3465,11 @@
         <v>67.7</v>
       </c>
       <c r="K4" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="L4" t="n">
-        <v>80.768</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>86.88500000000001</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; public-normal m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3496,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>k_1 (m20-m40 single-source) + public-normal (m50)</t>
+          <t>k_1 (m20-m40 single-source)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -3529,14 +3515,11 @@
         <v>94.04000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>86.02</v>
-      </c>
-      <c r="L5" t="n">
-        <v>94.215</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>result_wideband_pulse_png/rf_rgb/... for m20-m40; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m50</t>
+        <v>96.94670000000001</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>result_wideband_pulse_png/rf_rgb/... for m20-m40</t>
         </is>
       </c>
     </row>
@@ -3584,14 +3567,11 @@
         <v>85.6525</v>
       </c>
       <c r="K6" t="n">
-        <v>72.6375</v>
-      </c>
-      <c r="L6" t="n">
-        <v>89.43259999999999</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>aggregated from rows above</t>
+        <v>94.1011</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>aggregated from rows above; m50db retained only in supplementary records</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3662,15 +3642,10 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>m50db</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
         <is>
           <t>result_source</t>
         </is>
@@ -3699,12 +3674,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>optimized_spectral_gradient + rgb_fallback_m50db</t>
+          <t>optimized_spectral_gradient</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -3720,14 +3695,11 @@
         <v>84.31</v>
       </c>
       <c r="K2" t="n">
-        <v>60.46</v>
-      </c>
-      <c r="L2" t="n">
-        <v>86.91200000000001</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>93.52500000000001</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; optimized spectral gradient used at m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -3754,12 +3726,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>optimized_spectral_gradient + rgb_fallback_m50db</t>
+          <t>optimized_spectral_gradient</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -3775,14 +3747,11 @@
         <v>98.97</v>
       </c>
       <c r="K3" t="n">
-        <v>87.77</v>
-      </c>
-      <c r="L3" t="n">
-        <v>97.346</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>99.73999999999999</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; optimized spectral gradient used at m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -3809,12 +3778,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dsss_weak_residual + rgb_fallback_m50db</t>
+          <t>dsss_weak_residual</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -3830,14 +3799,11 @@
         <v>69.20999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="L4" t="n">
-        <v>81.13200000000001</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>87.34</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; dsss weak residual used at m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3830,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>k_1 (m20-m40 single-source) + public-normal (m50)</t>
+          <t>k_1 (m20-m40 single-source)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -3883,14 +3849,11 @@
         <v>94.04000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>86.02</v>
-      </c>
-      <c r="L5" t="n">
-        <v>94.215</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>result_wideband_pulse_png/rf_rgb/... for m20-m40; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m50</t>
+        <v>96.94670000000001</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>result_wideband_pulse_png/rf_rgb/... for m20-m40</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3885,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>selection_with_low_snr_fallback</t>
+          <t>morphology_aware_selection</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -3938,14 +3901,11 @@
         <v>86.63249999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>72.6375</v>
-      </c>
-      <c r="L6" t="n">
-        <v>90.1187</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>aggregated from rows above with optimized spectral gradient and m50db rgb fallback</t>
+        <v>94.3879</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>aggregated from rows above; m50db retained only in supplementary records</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4021,15 +3981,10 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>m50db</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t>result_source</t>
         </is>
@@ -4058,7 +4013,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4068,7 +4023,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>optimized_spectral_gradient + rgb_fallback_m50db</t>
+          <t>optimized_spectral_gradient</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -4084,14 +4039,11 @@
         <v>2.34</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>0.675</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; public-normal m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4070,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4128,7 +4080,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>optimized_spectral_gradient + rgb_fallback_m50db</t>
+          <t>optimized_spectral_gradient</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -4144,14 +4096,11 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>0.0175</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; public-normal m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4127,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>k_1 (legacy m10-m30) + public-normal (m40-m50)</t>
+          <t>k_1 (legacy m10-m30) + public-normal (m40)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4188,7 +4137,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>dsss_weak_residual + rgb_fallback_m50db</t>
+          <t>dsss_weak_residual</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -4204,14 +4153,11 @@
         <v>1.51</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.364</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>legacy rf_open for m10-m30; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m40-m50</t>
+        <v>0.455</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>legacy rf_open for m10-m30; public-normal m40 supplementary experiment</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4184,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>k_1 (m20-m40 single-source) + public-normal (m50)</t>
+          <t>k_1 (m20-m40 single-source)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4264,12 +4210,9 @@
       <c r="L5" t="n">
         <v>0</v>
       </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>result_wideband_pulse_png/rf_rgb/... for m20-m40; analysis_outputs/rf_spe_png_new_levels/new_m40_m50_baseline_vs_selected.csv for m50</t>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>result_wideband_pulse_png/rf_rgb/... for m20-m40</t>
         </is>
       </c>
     </row>
@@ -4306,7 +4249,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>selection_with_low_snr_fallback</t>
+          <t>morphology_aware_selection</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -4322,14 +4265,11 @@
         <v>0.98</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.6861</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>aggregated from rows above with optimized spectral gradient and m50db rgb fallback</t>
+        <v>0.2869</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>aggregated from rows above; m50db retained only in supplementary records</t>
         </is>
       </c>
     </row>

</xml_diff>